<commit_message>
Cases.xlsx and Check.xlsx changed
</commit_message>
<xml_diff>
--- a/Check.xlsx
+++ b/Check.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="66">
   <si>
     <t>Группа проверок/модуль</t>
   </si>
@@ -48,6 +48,12 @@
     <t>Вход с неверным паролем (login2/wrong) → отображается сообщение об ошибке ("Wrong login or password")</t>
   </si>
   <si>
+    <t>Не пройден</t>
+  </si>
+  <si>
+    <t>Появляется сообщение "Something went wrong. Try again later", а не "Wrong login or password", приложение не крашится.</t>
+  </si>
+  <si>
     <t>Вход с несуществующим логином → отображается сообщение об ошибке ("Wrong Login or Password")</t>
   </si>
   <si>
@@ -66,9 +72,6 @@
     <t>Переход между экранами через боковое меню: Main → News → About</t>
   </si>
   <si>
-    <t>Не пройден</t>
-  </si>
-  <si>
     <t>Main -&gt; News - переходит, а при переходе News -&gt; About - кнопка About неактивна.</t>
   </si>
   <si>
@@ -87,7 +90,7 @@
     <t>Новости</t>
   </si>
   <si>
-    <t>Отображение списка новостей (если новости есть) — каждая новость содержит заголовок, дату, категорию</t>
+    <t>Отображение списка новостей (если новости есть) — каждая новость содержит заголовок, дату, категорию, комментарий</t>
   </si>
   <si>
     <t>Создание новости со всеми заполненными полями (категория, заголовок, описание, дата, время) — новость появляется в списке</t>
@@ -126,7 +129,7 @@
     <t>Сортировка новостей по дате (от новых к старым) — порядок корректный</t>
   </si>
   <si>
-    <t>После создания новости дата создания в списке соответствует выбранной при создании</t>
+    <t>После создания новости дата создания в списке соответствует дате публикации</t>
   </si>
   <si>
     <t>Формат даты (день, месяц, год) и сама дата не соответствует той, что указывалась при создании</t>
@@ -171,13 +174,10 @@
     <t>Негативные сценарии</t>
   </si>
   <si>
-    <t>Попытка создать новость с датой в прошлом (если это запрещено логикой) — появляется ошибка</t>
-  </si>
-  <si>
-    <t>Попытка создать новость с датой в будущем (если это запрещено логикой) — появляется ошибка</t>
-  </si>
-  <si>
-    <t>Ошибка логики</t>
+    <t>Попытка создать новость с датой в прошлом  — нельзя выбрать дату раньше сегодняшней</t>
+  </si>
+  <si>
+    <t>Нельзя создать новость задним числом нельзя.</t>
   </si>
   <si>
     <t>Создание новости с пустым полем Category → сообщение об ошибке ("Fill empty fields")</t>
@@ -195,7 +195,10 @@
     <t>Создание новости с пустым полем Title → сообщение об ошибке ("Fill empty fields")</t>
   </si>
   <si>
-    <t>Создание новости с заголовком длиной 200+ символов → заголовок обрезается или переносится, приложение не крашится</t>
+    <t>Создание новости со всеми пустыми полями → сообщение об ошибке ("Fill empty fields")</t>
+  </si>
+  <si>
+    <t>Создание новости с заголовком длиной 50+ символов → заголовок обрезается или переносится, приложение не крашится</t>
   </si>
   <si>
     <t>Создание новости с HTML-тегами во всех полях (&lt;script&gt;alert(1)&lt;/script&gt;) → теги отображаются как обычный текст, скрипт не выполняется, новость не сохраняется, ошибка "Saving failed. Try again later"</t>
@@ -217,7 +220,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -236,12 +239,16 @@
     <font>
       <sz val="11.0"/>
       <color rgb="FF0F1115"/>
-      <name val="Quote-cjk-patch"/>
+      <name val="Arial"/>
     </font>
     <font/>
     <font>
-      <sz val="11.0"/>
-      <color rgb="FF0F1115"/>
+      <sz val="12.0"/>
+      <color rgb="FF0D0E11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -339,7 +346,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -372,17 +379,26 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="7" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="7" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="7" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="7" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -645,30 +661,34 @@
         <v>7</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11"/>
       <c r="B4" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="E4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="10"/>
     </row>
     <row r="5">
       <c r="A5" s="11"/>
       <c r="B5" s="12" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>8</v>
@@ -676,9 +696,9 @@
       <c r="E5" s="10"/>
     </row>
     <row r="6">
-      <c r="A6" s="13"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>7</v>
@@ -690,28 +710,28 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>17</v>
+        <v>10</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11"/>
       <c r="B8" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>8</v>
@@ -721,10 +741,10 @@
     <row r="9">
       <c r="A9" s="11"/>
       <c r="B9" s="12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>8</v>
@@ -732,12 +752,12 @@
       <c r="E9" s="10"/>
     </row>
     <row r="10">
-      <c r="A10" s="13"/>
+      <c r="A10" s="14"/>
       <c r="B10" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="9" t="s">
         <v>21</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>20</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>8</v>
@@ -746,10 +766,10 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>7</v>
@@ -762,7 +782,7 @@
     <row r="12">
       <c r="A12" s="11"/>
       <c r="B12" s="12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>7</v>
@@ -775,22 +795,22 @@
     <row r="13">
       <c r="A13" s="11"/>
       <c r="B13" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>26</v>
+        <v>10</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11"/>
       <c r="B14" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>7</v>
@@ -803,10 +823,10 @@
     <row r="15">
       <c r="A15" s="11"/>
       <c r="B15" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>8</v>
@@ -816,10 +836,10 @@
     <row r="16">
       <c r="A16" s="11"/>
       <c r="B16" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D16" s="9" t="s">
         <v>8</v>
@@ -829,10 +849,10 @@
     <row r="17">
       <c r="A17" s="11"/>
       <c r="B17" s="12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>8</v>
@@ -842,10 +862,10 @@
     <row r="18">
       <c r="A18" s="11"/>
       <c r="B18" s="12" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>8</v>
@@ -855,10 +875,10 @@
     <row r="19">
       <c r="A19" s="11"/>
       <c r="B19" s="12" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>8</v>
@@ -868,10 +888,10 @@
     <row r="20">
       <c r="A20" s="11"/>
       <c r="B20" s="12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>8</v>
@@ -881,10 +901,10 @@
     <row r="21">
       <c r="A21" s="11"/>
       <c r="B21" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>8</v>
@@ -893,39 +913,39 @@
     </row>
     <row r="22">
       <c r="A22" s="11"/>
-      <c r="B22" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="10"/>
+      <c r="B22" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="17"/>
     </row>
     <row r="23">
       <c r="A23" s="11"/>
       <c r="B23" s="12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13"/>
+      <c r="A24" s="14"/>
       <c r="B24" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>8</v>
@@ -934,10 +954,10 @@
     </row>
     <row r="25">
       <c r="A25" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>7</v>
@@ -950,10 +970,10 @@
     <row r="26">
       <c r="A26" s="11"/>
       <c r="B26" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>8</v>
@@ -961,12 +981,12 @@
       <c r="E26" s="10"/>
     </row>
     <row r="27">
-      <c r="A27" s="13"/>
+      <c r="A27" s="14"/>
       <c r="B27" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>8</v>
@@ -975,10 +995,10 @@
     </row>
     <row r="28">
       <c r="A28" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>7</v>
@@ -990,86 +1010,86 @@
     </row>
     <row r="29">
       <c r="A29" s="11"/>
-      <c r="B29" s="15" t="s">
-        <v>45</v>
+      <c r="B29" s="18" t="s">
+        <v>46</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>46</v>
+        <v>10</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11"/>
-      <c r="B30" s="16" t="s">
+      <c r="B30" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>46</v>
-      </c>
     </row>
     <row r="31">
-      <c r="A31" s="13"/>
-      <c r="B31" s="16" t="s">
-        <v>48</v>
+      <c r="A31" s="14"/>
+      <c r="B31" s="19" t="s">
+        <v>49</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E31" s="14" t="s">
-        <v>49</v>
+        <v>10</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="16" t="s">
         <v>51</v>
       </c>
+      <c r="B32" s="19" t="s">
+        <v>52</v>
+      </c>
       <c r="C32" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E32" s="10"/>
+      <c r="E32" s="13" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="11"/>
-      <c r="B33" s="16" t="s">
-        <v>52</v>
+      <c r="B33" s="12" t="s">
+        <v>54</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D33" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E33" s="14" t="s">
-        <v>53</v>
-      </c>
+      <c r="E33" s="10"/>
     </row>
     <row r="34">
       <c r="A34" s="11"/>
       <c r="B34" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D34" s="9" t="s">
         <v>8</v>
@@ -1079,10 +1099,10 @@
     <row r="35">
       <c r="A35" s="11"/>
       <c r="B35" s="12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D35" s="9" t="s">
         <v>8</v>
@@ -1092,10 +1112,10 @@
     <row r="36">
       <c r="A36" s="11"/>
       <c r="B36" s="12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D36" s="9" t="s">
         <v>8</v>
@@ -1105,10 +1125,10 @@
     <row r="37">
       <c r="A37" s="11"/>
       <c r="B37" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>8</v>
@@ -1118,10 +1138,10 @@
     <row r="38">
       <c r="A38" s="11"/>
       <c r="B38" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>8</v>
@@ -1131,10 +1151,10 @@
     <row r="39">
       <c r="A39" s="11"/>
       <c r="B39" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D39" s="9" t="s">
         <v>8</v>
@@ -1142,12 +1162,12 @@
       <c r="E39" s="10"/>
     </row>
     <row r="40">
-      <c r="A40" s="13"/>
+      <c r="A40" s="14"/>
       <c r="B40" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D40" s="9" t="s">
         <v>8</v>
@@ -1156,28 +1176,28 @@
     </row>
     <row r="41">
       <c r="A41" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B41" s="16" t="s">
         <v>62</v>
       </c>
+      <c r="B41" s="19" t="s">
+        <v>63</v>
+      </c>
       <c r="C41" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>63</v>
+        <v>10</v>
+      </c>
+      <c r="E41" s="13" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13"/>
-      <c r="B42" s="16" t="s">
-        <v>64</v>
+      <c r="A42" s="14"/>
+      <c r="B42" s="19" t="s">
+        <v>65</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>8</v>
@@ -1190,8 +1210,8 @@
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="A25:A27"/>
     <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A41:A42"/>
     <mergeCell ref="A11:A24"/>
-    <mergeCell ref="A41:A42"/>
     <mergeCell ref="A32:A40"/>
   </mergeCells>
   <dataValidations>

</xml_diff>